<commit_message>
chore(data): name real suppliers — Tomike (Ondo) + Daniela PNC Tropical Foods
Mary confirmed:
- Jan/Feb purchases were from "Tomike from Ondo"
- Mar purchases (the ones previously labelled "Prime Foods" / "Prime Fruits")
  were from "Daniela PNC Tropical Foods"
- Feb 10 discrepancy resolved: trusted the stated 315k total (= 45k/keg)

Updates seed.ts, seed-real-data.sql, build_ledger.py, and refreshes
data/cyfoods-ledger.xlsx. Open-questions sheet trimmed to the 3 still
outstanding (logistics-attribution, prior keg movements, missing entries).

Live DB updated via UPDATE on the two existing supplier rows — no destructive
re-seed needed.
</commit_message>
<xml_diff>
--- a/data/cyfoods-ledger.xlsx
+++ b/data/cyfoods-ledger.xlsx
@@ -582,7 +582,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Unspecified Supplier</t>
+          <t>Tomike from Ondo</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
@@ -625,7 +625,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Unspecified Supplier</t>
+          <t>Tomike from Ondo</t>
         </is>
       </c>
       <c r="C6" s="5" t="n">
@@ -656,7 +656,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Source said '47k each' but stated total 315k implies 45k. Trusted total.</t>
+          <t>Stated total 315k confirmed (315/7 = 45k/keg).</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Unspecified Supplier</t>
+          <t>Tomike from Ondo</t>
         </is>
       </c>
       <c r="C7" s="5" t="n">
@@ -707,7 +707,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Unspecified Supplier</t>
+          <t>Tomike from Ondo</t>
         </is>
       </c>
       <c r="C8" s="5" t="n">
@@ -750,7 +750,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Prime Foods</t>
+          <t>Daniela PNC Tropical Foods</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
@@ -789,7 +789,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Prime Foods</t>
+          <t>Daniela PNC Tropical Foods</t>
         </is>
       </c>
       <c r="C10" s="5" t="n">
@@ -1023,7 +1023,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Prime Foods</t>
+          <t>Daniela PNC Tropical Foods</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
@@ -1033,7 +1033,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Unspecified Supplier</t>
+          <t>Tomike from Ondo</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
@@ -1055,7 +1055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>What's the supplier for the Jan 19 / Feb 10 / Feb 11 / Feb 16 purchases? (Currently grouped under 'Unspecified Supplier'.)</t>
+          <t>Logistics: '20 rubbers @ 4k each' was applied to the 20-keg Feb 16 load (Tomike). '10 rubbers @ 6k each' was applied to Mar 19 (Daniela PNC). Confirm — could it have applied to Feb 11 instead?</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Feb 10 had a discrepancy: '47k per keg' but '315k total for 7'. We trusted the total (= 45k/keg). Confirm which is right.</t>
+          <t>Were any of these kegs sold, packed, or repackaged before today? (Currently we assume all 57 kegs are still on hand.)</t>
         </is>
       </c>
     </row>
@@ -1112,30 +1112,6 @@
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Logistics: '20 rubbers @ 4k each' was applied to the 20-keg Feb 16 load. '10 rubbers @ 6k each' was applied to Mar 19 (Prime Foods). Confirm — could it have applied to Feb 11 instead?</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Were any of these kegs sold, packed, or repackaged before today? (Currently we assume all 57 kegs are still on hand.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Q5</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Any other purchases between Jan 19 and Mar 19, or after Mar 19, that aren't on this list?</t>
         </is>

</xml_diff>